<commit_message>
Rechner: Abgleich mit PDF des DIW aktuell Nr. 126
- Marke 21 Mrd.: Schwelle, ab der bei 8 Euro Miete Zuschüsse nötig sind
- 8-Euro-Miete und IMK-Hinweis wie im DIW aktuell begründet
- ISSN ergänzt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -381,7 +381,7 @@
     <t xml:space="preserve">Nettokaltmiete im ersten Jahr</t>
   </si>
   <si>
-    <t xml:space="preserve">4,04 Faire-Mieten-Modell (Holm et al. 2025) · 6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø landeseigene Unternehmen 2025 (7,11; DIW aktuell Nr. 126), Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (7,94 Ende 2023, Bernt/Holm 2023).</t>
+    <t xml:space="preserve">4,04 Faire-Mieten-Modell (Holm et al. 2025) · 6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø landeseigene Unternehmen 2025 (7,11; DIW aktuell Nr. 126), Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (DIW aktuell Nr. 126 nach Geschäftsberichten von Adler, Grand City Properties, Vonovia).</t>
   </si>
   <si>
     <t xml:space="preserve">Mietsteigerung pro Jahr</t>
@@ -618,7 +618,7 @@
     <t xml:space="preserve">Quellen</t>
   </si>
   <si>
-    <t xml:space="preserve">Dany-Knedlik, G., Kholodilin, K. A., Kritikos, A. S., Kriwoluzky, A. (2026): Vergesellschaftung der Wohnungsunternehmen in Berlin belastet den Haushalt und schafft keine zusätzliche Wohnung. DIW aktuell Nr. 126, 5.10.2026. https://www.diw.de/de/diw_01.c.1021274.de/publikationen/diw_aktuell/2026_0126/vergesellschaftung_der_wohnungsunternehmen_in_berlin_belastet_den_haushalt_und_schafft_keine_zusaetzliche_wohnung.html</t>
+    <t xml:space="preserve">Dany-Knedlik, G., Kholodilin, K. A., Kritikos, A. S., Kriwoluzky, A. (2026): Vergesellschaftung der Wohnungsunternehmen in Berlin belastet den Haushalt und schafft keine zusätzliche Wohnung. DIW aktuell Nr. 126, 5.10.2026, ISSN 2567-3971. https://www.diw.de/de/diw_01.c.1021274.de/publikationen/diw_aktuell/2026_0126/vergesellschaftung_der_wohnungsunternehmen_in_berlin_belastet_den_haushalt_und_schafft_keine_zusaetzliche_wohnung.html</t>
   </si>
   <si>
     <t xml:space="preserve">Dullien, S., Kaczmarczyk, P., Krebs, T., Truger, A. (2026): Die Überführung von großen Wohnungsbeständen ins Gemeineigentum. IMK Policy Brief Nr. 225.</t>
@@ -2496,7 +2496,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
         <v>103</v>
       </c>

</xml_diff>

<commit_message>
Rechner: Link und Zitation DIW aktuell Nr. 126, Angleichung an veröffentlichte Fassung
- Verweise auf DIW aktuell Nr. 126 (5.10.2026) mit Link
- Tabelle 2 statt 2a/2b; Zins +1 Pp. als Sensitivität gekennzeichnet
- Haushaltsausgaben 2027: bereinigt 45,9 Mrd. Euro wie im DIW aktuell
- 7 Euro: Durchschnitt landeseigene Unternehmen 2025 (7,11 Euro)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="195">
   <si>
     <t xml:space="preserve">Was kostet die Vergesellschaftung den Berliner Landeshaushalt?</t>
   </si>
@@ -78,7 +78,10 @@
     <t xml:space="preserve">Grundlage</t>
   </si>
   <si>
-    <t xml:space="preserve">DIW aktuell „Vergesellschaftung in Berlin: Teuer für den Haushalt, keine zusätzliche Wohnung“ (Dany-Knedlik, Kholodilin, Kritikos, Kriwoluzky, 2026), Tabelle 2.</t>
+    <t xml:space="preserve">Dany-Knedlik, Kholodilin, Kritikos, Kriwoluzky (2026): „Vergesellschaftung der Wohnungsunternehmen in Berlin belastet den Haushalt und schafft keine zusätzliche Wohnung“. DIW aktuell Nr. 126, 5.10.2026, Tabelle 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.diw.de/de/diw_01.c.1021274.de/publikationen/diw_aktuell/2026_0126/vergesellschaftung_der_wohnungsunternehmen_in_berlin_belastet_den_haushalt_und_schafft_keine_zusaetzliche_wohnung.html</t>
   </si>
   <si>
     <t xml:space="preserve">Rechenlogik</t>
@@ -102,7 +105,7 @@
     <t xml:space="preserve">3. „Ergebnis“ zeigt die Kennzahlen und die Einordnung in den Landeshaushalt, „Zeitreihe“ die Rechnung Jahr für Jahr, „Matrix“ die Belastung im ersten Jahr für mehrere Entschädigungen und Mieten (wie Tabelle 2 im DIW aktuell).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Die DIW-Tabelle 2a erhalten Sie mit den Standardwerten (Zinsen 4 % / 5 %). Das erste Jahr hängt nicht von Miet- und Kostensteigerung ab; setzt man beide auf 0 %, ist die Belastung in allen Jahren gleich hoch.</t>
+    <t xml:space="preserve">4. Tabelle 2 des DIW aktuell erhalten Sie mit den Standardwerten (Zinsen 4 % / 5 %). Das erste Jahr hängt nicht von Miet- und Kostensteigerung ab; setzt man beide auf 0 %, ist die Belastung in allen Jahren gleich hoch.</t>
   </si>
   <si>
     <t xml:space="preserve">Farblegende</t>
@@ -192,7 +195,7 @@
     <t xml:space="preserve">Einordnung der Belastung im ersten Jahr</t>
   </si>
   <si>
-    <t xml:space="preserve">in % des Haushaltsvolumens 2027</t>
+    <t xml:space="preserve">in % der bereinigten Ausgaben 2027</t>
   </si>
   <si>
     <t xml:space="preserve">%</t>
@@ -315,7 +318,7 @@
     <t xml:space="preserve">Matrix: Belastung im ersten Jahr nach Entschädigung und Miete</t>
   </si>
   <si>
-    <t xml:space="preserve">Zinsen, Eigenkapitalquote, Laufzeiten, Bestand und Bewirtschaftungskosten aus dem Blatt „Annahmen“. Mit den Standardwerten entspricht das Tabelle 2a im DIW aktuell. Zeilen- und Spaltenköpfe (blau) sind änderbar.</t>
+    <t xml:space="preserve">Zinsen, Eigenkapitalquote, Laufzeiten, Bestand und Bewirtschaftungskosten aus dem Blatt „Annahmen“. Mit den Standardwerten entspricht das Tabelle 2 im DIW aktuell Nr. 126. Zeilen- und Spaltenköpfe (blau) sind änderbar.</t>
   </si>
   <si>
     <t xml:space="preserve">Kapitaldienst je Mrd. € Entschädigung (Mio. € pro Jahr)</t>
@@ -378,7 +381,7 @@
     <t xml:space="preserve">Nettokaltmiete im ersten Jahr</t>
   </si>
   <si>
-    <t xml:space="preserve">4,04 Faire-Mieten-Modell (Holm et al. 2025) · 6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (7,94 Ende 2023, Bernt/Holm 2023).</t>
+    <t xml:space="preserve">4,04 Faire-Mieten-Modell (Holm et al. 2025) · 6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø landeseigene Unternehmen 2025 (7,11; DIW aktuell Nr. 126), Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (7,94 Ende 2023, Bernt/Holm 2023).</t>
   </si>
   <si>
     <t xml:space="preserve">Mietsteigerung pro Jahr</t>
@@ -420,7 +423,7 @@
     <t xml:space="preserve">Zins auf die Kredite der Anstalt</t>
   </si>
   <si>
-    <t xml:space="preserve">Bundesanleihen mittlerer Laufzeit ≈ 3,3 % (Bundesbank, 20.10.2026) + rund 1 Prozentpunkt Aufschlag (HOWOGE-Anleihe, 7 J. Restlaufzeit); 5 % vorsichtig gerundet. Holm et al. (2025): +1,5 bis +2,0 Prozentpunkte. DIW Tabelle 2b: Zinsen jeweils +1 Pp.</t>
+    <t xml:space="preserve">Bundesanleihen mittlerer Laufzeit ≈ 3,3 % (Bundesbank, 20.10.2026) + rund 1 Prozentpunkt Aufschlag (HOWOGE-Anleihe, 7 J. Restlaufzeit); 5 % vorsichtig gerundet. Holm et al. (2025): +1,5 bis +2,0 Prozentpunkte. Sensitivität: Zinsen jeweils +1 Pp.</t>
   </si>
   <si>
     <t xml:space="preserve">Laufzeit Eigenkapital-Kredit</t>
@@ -522,10 +525,10 @@
     <t xml:space="preserve">Quelle</t>
   </si>
   <si>
-    <t xml:space="preserve">Haushaltsvolumen 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doppelhaushalt 2026/27 (beschlossen 18.12.2025); 2026: ≈ 45,5 Mrd. €</t>
+    <t xml:space="preserve">Bereinigte Ausgaben des Landes 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doppelhaushalt 2026/27, Pressemitteilung SenFin Nr. 21 vom 19.12.2025; 2026: knapp 45 Mrd. € (wie DIW aktuell Nr. 126)</t>
   </si>
   <si>
     <t xml:space="preserve">Finanzierungsdefizit 2026</t>
@@ -615,7 +618,7 @@
     <t xml:space="preserve">Quellen</t>
   </si>
   <si>
-    <t xml:space="preserve">Dany-Knedlik, G., Kholodilin, K. A., Kritikos, A. S., Kriwoluzky, A. (2026): Vergesellschaftung in Berlin: Teuer für den Haushalt, keine zusätzliche Wohnung. DIW aktuell.</t>
+    <t xml:space="preserve">Dany-Knedlik, G., Kholodilin, K. A., Kritikos, A. S., Kriwoluzky, A. (2026): Vergesellschaftung der Wohnungsunternehmen in Berlin belastet den Haushalt und schafft keine zusätzliche Wohnung. DIW aktuell Nr. 126, 5.10.2026. https://www.diw.de/de/diw_01.c.1021274.de/publikationen/diw_aktuell/2026_0126/vergesellschaftung_der_wohnungsunternehmen_in_berlin_belastet_den_haushalt_und_schafft_keine_zusaetzliche_wohnung.html</t>
   </si>
   <si>
     <t xml:space="preserve">Dullien, S., Kaczmarczyk, P., Krebs, T., Truger, A. (2026): Die Überführung von großen Wohnungsbeständen ins Gemeineigentum. IMK Policy Brief Nr. 225.</t>
@@ -1328,7 +1331,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:B24"/>
+  <dimension ref="B1:B25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1358,38 +1361,38 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="3"/>
+    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="3" t="s">
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="3"/>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="s">
-        <v>7</v>
-      </c>
+      <c r="B11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
@@ -1404,43 +1407,48 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="3"/>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="3" t="s">
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="3"/>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="B20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="3"/>
+      <c r="B22" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="3" t="s">
+      <c r="B23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1472,470 +1480,470 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">Zeitreihe!K5</f>
         <v>142.800684459716</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">Zeitreihe!L5</f>
         <v>0.812845426114048</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">Zeitreihe!M5</f>
         <v>49.5835709929569</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="15" t="n">
         <f aca="false">Zeitreihe!G5</f>
         <v>574.4736</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C9" s="15" t="n">
         <f aca="false">Zeitreihe!H5</f>
         <v>125.685541213762</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" s="15" t="n">
         <f aca="false">Zeitreihe!I5</f>
         <v>591.588743245954</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" s="15" t="n">
         <f aca="false">Zeitreihe!O5</f>
         <v>-17.1151432459538</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" s="16" t="n">
         <f aca="false">B1/HH_Ausgaben</f>
-        <v>0.00307098246149927</v>
+        <v>0.00311112602308749</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E14" s="13"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" s="16" t="n">
         <f aca="false">B1/HH_Defizit</f>
         <v>0.03104362705646</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" s="16" t="n">
         <f aca="false">B1/HH_EP10</f>
         <v>0.0262984685929495</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="17" t="n">
         <f aca="false">B1/HH_Spielraum</f>
         <v>0.178500855574645</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E17" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C20" s="18" t="n">
         <f aca="false">Horizont</f>
         <v>50</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C21" s="15" t="n">
         <f aca="false">SUMIF(Z_Belastung,"&gt;0")</f>
         <v>12013.2027926495</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C22" s="15" t="n">
         <f aca="false">SUM(Z_Belastung)</f>
         <v>12013.2027926495</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C23" s="15" t="n">
         <f aca="false">SUM(Z_Barwert)</f>
         <v>4258.15411069692</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C24" s="15" t="n">
         <f aca="false">INDEX(Z_Belastung,Horizont)</f>
         <v>443.974112005765</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C25" s="15" t="n">
         <f aca="false">MAX(0,MAX(Z_Kum))</f>
         <v>12013.2027926495</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C26" s="18" t="n">
         <f aca="false">COUNT(Z_MitZuschuss)</f>
         <v>50</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C27" s="18" t="str">
         <f aca="false">IF(COUNT(Z_MitZuschuss)=0,1,IF(MAX(Z_MitZuschuss)&gt;=Horizont,"nicht im Zeitraum",MAX(Z_MitZuschuss)+1))</f>
         <v>nicht im Zeitraum</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C28" s="19" t="n">
         <f aca="false">INDEX(Z_RestEK,Horizont)+INDEX(Z_RestFK,Horizont)</f>
         <v>0</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E28" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C31" s="19" t="n">
         <f aca="false">Eigenkapital</f>
         <v>2700</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C32" s="20" t="n">
         <f aca="false">Eigenkapital/HH_Schulden</f>
         <v>0.0391304347826087</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C33" s="19" t="n">
         <f aca="false">Fremdkapital</f>
         <v>10800</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C36" s="21" t="n">
         <f aca="false">MAX(0,Zeitreihe!G5)/1000/(EK_Quote*IF(Nur_Zinsen=1,Zins_EK,AF_EK)+(1-EK_Quote)*IF(Nur_Zinsen=1,Zins_FK,AF_FK))</f>
         <v>10.8123123441428</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C37" s="22" t="n">
         <f aca="false">Bewirtschaftung+Zeitreihe!J5*1000000/Flaeche/12</f>
         <v>7.81284542611405</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C40" s="23" t="n">
         <f aca="false">IF(Nur_Zinsen=1,Zins_FK/Marktrendite,AF_FK/IF(Marktrendite=0,1/Laufzeit_FK,Marktrendite/(1-(1+Marktrendite)^(-Laufzeit_FK))))</f>
         <v>1.15684359846251</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1964,12 +1972,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1980,7 +1988,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C5" s="25" t="n">
         <f aca="false">1000*(EK_Quote*IF(Nur_Zinsen=1,Zins_EK,AF_EK)+(1-EK_Quote)*IF(Nur_Zinsen=1,Zins_FK,AF_FK))</f>
@@ -1989,12 +1997,12 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>4.04</v>
@@ -2164,12 +2172,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C17" s="31" t="n">
         <f aca="false">C8</f>
@@ -2350,12 +2358,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="34" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C26" s="34"/>
       <c r="D26" s="34"/>
@@ -2412,34 +2420,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C5" s="35" t="n">
         <v>13.5</v>
@@ -2448,15 +2456,15 @@
         <v>13.5</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C6" s="38" t="n">
         <v>240000</v>
@@ -2465,15 +2473,15 @@
         <v>240000</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" s="38" t="n">
         <v>61</v>
@@ -2482,15 +2490,15 @@
         <v>61</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C8" s="40" t="n">
         <v>7</v>
@@ -2499,15 +2507,15 @@
         <v>7</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C9" s="42" t="n">
         <v>0.01</v>
@@ -2516,15 +2524,15 @@
         <v>0.01</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C10" s="44" t="n">
         <v>3.73</v>
@@ -2533,15 +2541,15 @@
         <v>3.73</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C11" s="45" t="n">
         <v>0.02</v>
@@ -2550,15 +2558,15 @@
         <v>0.02</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C12" s="45" t="n">
         <v>0.2</v>
@@ -2567,15 +2575,15 @@
         <v>0.2</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C13" s="46" t="n">
         <v>0.04</v>
@@ -2584,15 +2592,15 @@
         <v>0.04</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="12" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C14" s="46" t="n">
         <v>0.05</v>
@@ -2601,15 +2609,15 @@
         <v>0.05</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C15" s="48" t="n">
         <v>50</v>
@@ -2618,15 +2626,15 @@
         <v>50</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F15" s="37" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="12" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C16" s="48" t="n">
         <v>50</v>
@@ -2635,32 +2643,32 @@
         <v>50</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="12" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F17" s="37" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C18" s="48" t="n">
         <v>50</v>
@@ -2669,28 +2677,28 @@
         <v>50</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C19" s="52"/>
       <c r="D19" s="47"/>
       <c r="E19" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F19" s="37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C20" s="52" t="n">
         <v>0.041</v>
@@ -2699,80 +2707,80 @@
         <v>0.041</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="26" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C24" s="19" t="n">
         <f aca="false">Wohnungen*Flaeche_je_WE</f>
         <v>14640000</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C25" s="19" t="n">
         <f aca="false">EK_Quote*Entschaedigung*1000</f>
         <v>2700</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C26" s="19" t="n">
         <f aca="false">(1-EK_Quote)*Entschaedigung*1000</f>
         <v>10800</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C27" s="18" t="n">
         <f aca="false">IF(Tilgung="nur Zinsen",1,0)</f>
@@ -2783,7 +2791,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C28" s="53" t="n">
         <f aca="false">IF(Zins_EK=0,1/Laufzeit_EK,Zins_EK/(1-(1+Zins_EK)^(-Laufzeit_EK)))</f>
@@ -2791,12 +2799,12 @@
       </c>
       <c r="E28" s="12"/>
       <c r="F28" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C29" s="53" t="n">
         <f aca="false">IF(Zins_FK=0,1/Laufzeit_FK,Zins_FK/(1-(1+Zins_FK)^(-Laufzeit_FK)))</f>
@@ -2804,142 +2812,142 @@
       </c>
       <c r="E29" s="12"/>
       <c r="F29" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C30" s="21" t="n">
         <f aca="false">Eigenkapital*IF(Nur_Zinsen=1,Zins_EK,AF_EK)</f>
         <v>125.685541213762</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C31" s="21" t="n">
         <f aca="false">Fremdkapital*IF(Nur_Zinsen=1,Zins_FK,AF_FK)</f>
         <v>591.588743245954</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C32" s="54" t="n">
         <f aca="false">IF(ISBLANK(Diskont_Eingabe),Zins_EK,Diskont_Eingabe)</f>
         <v>0.04</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C36" s="38" t="n">
-        <v>46500</v>
+        <v>45900</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F36" s="37" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C37" s="38" t="n">
         <v>4600</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F37" s="37" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C38" s="38" t="n">
         <v>5430</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F38" s="37" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C39" s="38" t="n">
         <v>800</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F39" s="37" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C40" s="38" t="n">
         <v>69000</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F40" s="37" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -2993,74 +3001,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="55" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B4" s="55" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C4" s="55" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D4" s="55" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E4" s="55" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F4" s="55" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G4" s="55" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H4" s="55" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I4" s="55" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J4" s="55" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K4" s="55" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L4" s="55" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="M4" s="55" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N4" s="55" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="O4" s="55" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P4" s="55" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="Q4" s="55" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="R4" s="55" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="S4" s="55" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="T4" s="55" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11287,67 +11295,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rechner: Kostensteigerung fest 2 % (EZB-Inflationsziel), Mietsteigerung Standard 1 %
- Regler für die Kostensteigerung entfernt; 2 % p.a. fest, auch bei alten Links
- Mietsteigerung 1 % als politisch debattierter Wert begründet
- IMK-Voreinstellung: Mieten +2 % (real konstant wie beim IMK)
- Excel: Kostensteigerung als feste Annahme gekennzeichnet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -105,7 +105,7 @@
     <t xml:space="preserve">3. „Ergebnis“ zeigt die Kennzahlen und die Einordnung in den Landeshaushalt, „Zeitreihe“ die Rechnung Jahr für Jahr, „Matrix“ den Saldo im ersten Jahr für mehrere Entschädigungen und Mieten (wie Tabelle 2 im DIW aktuell, dort mit umgekehrtem Vorzeichen).</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Tabelle 2 des DIW aktuell erhalten Sie mit den Standardwerten (Zinsen 4 % / 5 %). Das erste Jahr hängt nicht von Miet- und Kostensteigerung ab; setzt man beide auf 0 %, ist der Saldo in allen Jahren gleich hoch.</t>
+    <t xml:space="preserve">4. Mit den Standardwerten entspricht das erste Jahr Tabelle 2 im DIW aktuell (13,5 Mrd. €, 7 € Miete). Ab dem zweiten Jahr steigen die Mieten um 1 % pro Jahr (änderbar) und die Bewirtschaftungskosten fest um 2 % pro Jahr, das Inflationsziel der EZB.</t>
   </si>
   <si>
     <t xml:space="preserve">Farblegende</t>
@@ -390,7 +390,7 @@
     <t xml:space="preserve">% p.a.</t>
   </si>
   <si>
-    <t xml:space="preserve">Holm et al. (2025), Grundmodell 1 % p.a.; Wahlprogramm Die Linke: LWU-Mieterhöhungen max. 1 % p.a.</t>
+    <t xml:space="preserve">Ab dem zweiten Jahr. 1 % wie politisch debattiert (Wahlprogramm Die Linke Berlin 2026: Mieterhöhungen der LWU max. 1 % p.a.; auch Holm et al. 2025, Grundmodell).</t>
   </si>
   <si>
     <t xml:space="preserve">Bewirtschaftungskosten im ersten Jahr</t>
@@ -399,10 +399,10 @@
     <t xml:space="preserve">Holm et al. (2025), Tab. 5 (LWU): Instandhaltung 1,77 + Modernisierung 1,00 + Verwaltung 0,52 + Mietausfallwagnis 0,14 + nicht umlagefähige Betriebskosten 0,30. Alternativen: 2,94 (Holm Basis), 3,66 (IMK), 4,40 (IW Köln), 4,44 (Holm Plus).</t>
   </si>
   <si>
-    <t xml:space="preserve">Kostensteigerung pro Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holm et al. (2025): inflationsbedingt 2 % p.a.</t>
+    <t xml:space="preserve">Kostensteigerung pro Jahr (fest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fest: Inflationsziel der EZB. Im Online-Rechner nicht veränderbar.</t>
   </si>
   <si>
     <t xml:space="preserve">Eigenkapitalquote (Land, kreditfinanziert)</t>
@@ -2516,7 +2516,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="12" t="s">
         <v>105</v>
       </c>
@@ -2554,7 +2554,7 @@
       <c r="B11" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="C11" s="45" t="n">
+      <c r="C11" s="20" t="n">
         <v>0.02</v>
       </c>
       <c r="D11" s="43" t="n">

</xml_diff>

<commit_message>
Rechner: Voreinstellung Sondierung Linke/Grüne/SPD (16 Mrd. Euro, 160.000 Wohnungen)
Miete 8,26 Euro (heutiges Niveau laut Vonovia), übrige Annahmen wie im
DIW aktuell. Quelle: dpa-Bericht vom 21.10.2026 zum Sondierungspapier.
Marke 16 Mrd. am Entschädigungsregler, Zeile in Tabelle und Excel-Matrix.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -344,7 +344,7 @@
     <t xml:space="preserve">Entschädigung</t>
   </si>
   <si>
-    <t xml:space="preserve">Spannweite der Schätzungen 8–36 Mrd. €: Initiative DWE 8/11; Holm et al. (2025) 10,1 (realitätsnah 10–17); IMK (2026) 13,5; Rechnungshof Berlin (2024) 8/11/29/36; Senat (2019/20) Verkehrswert 29–36 (bis 39,5).</t>
+    <t xml:space="preserve">Spannweite der Schätzungen 8–36 Mrd. €: Initiative DWE 8/11; Holm et al. (2025) 10,1 (realitätsnah 10–17); IMK (2026) 13,5; Sondierungspapier Linke/Grüne/SPD (Okt. 2026) Obergrenze 16 für rund 160.000 Wohnungen; Rechnungshof Berlin (2024) 8/11/29/36; Senat (2019/20) Verkehrswert 29–36 (bis 39,5).</t>
   </si>
   <si>
     <t xml:space="preserve">Zahl der Wohnungen</t>
@@ -353,7 +353,7 @@
     <t xml:space="preserve">Wohnungen</t>
   </si>
   <si>
-    <t xml:space="preserve">Rechnungshof Berlin (2024), Holm et al. (2025). Alternative IMK / DWE-Gesetzentwurf 2025: 210.000.</t>
+    <t xml:space="preserve">Rechnungshof Berlin (2024), Holm et al. (2025). Alternativen: IMK / DWE-Gesetzentwurf 2025: 210.000; Sondierungspapier Linke/Grüne/SPD 2026: rund 160.000 (Unternehmen &gt; 10.000 Wohnungen).</t>
   </si>
   <si>
     <t xml:space="preserve">Ø Wohnfläche je Wohnung</t>
@@ -2047,76 +2047,101 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="28" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C12" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-1061.29919804845</v>
+        <v>-795.64205565596</v>
       </c>
       <c r="D12" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-716.966398048447</v>
+        <v>-451.30925565596</v>
       </c>
       <c r="E12" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-541.286398048447</v>
+        <v>-275.62925565596</v>
       </c>
       <c r="F12" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-365.606398048447</v>
+        <v>-99.9492556559599</v>
       </c>
       <c r="G12" s="29" t="n">
         <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-189.926398048447</v>
+        <v>75.7307443440403</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="28" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C13" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-1486.35062587643</v>
+        <v>-1061.29919804845</v>
       </c>
       <c r="D13" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-1142.01782587643</v>
+        <v>-716.966398048447</v>
       </c>
       <c r="E13" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-966.337825876427</v>
+        <v>-541.286398048447</v>
       </c>
       <c r="F13" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-790.657825876427</v>
+        <v>-365.606398048447</v>
       </c>
       <c r="G13" s="29" t="n">
         <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-614.977825876427</v>
+        <v>-189.926398048447</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="28" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C14" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-1858.27062522591</v>
+        <v>-1486.35062587643</v>
       </c>
       <c r="D14" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-1513.93782522591</v>
+        <v>-1142.01782587643</v>
       </c>
       <c r="E14" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-1338.25782522591</v>
+        <v>-966.337825876427</v>
       </c>
       <c r="F14" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-1162.57782522591</v>
+        <v>-790.657825876427</v>
       </c>
       <c r="G14" s="29" t="n">
         <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
+        <v>-614.977825876427</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="28" t="n">
+        <v>36</v>
+      </c>
+      <c r="C15" s="29" t="n">
+        <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
+        <v>-1858.27062522591</v>
+      </c>
+      <c r="D15" s="29" t="n">
+        <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
+        <v>-1513.93782522591</v>
+      </c>
+      <c r="E15" s="29" t="n">
+        <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
+        <v>-1338.25782522591</v>
+      </c>
+      <c r="F15" s="29" t="n">
+        <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
+        <v>-1162.57782522591</v>
+      </c>
+      <c r="G15" s="29" t="n">
+        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
         <v>-986.897825225909</v>
       </c>
     </row>
@@ -2231,78 +2256,104 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="31" t="n">
         <f aca="false">B12</f>
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C21" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-6.0410928850663</v>
+        <v>-4.52892791243147</v>
       </c>
       <c r="D21" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-4.0810928850663</v>
+        <v>-2.56892791243146</v>
       </c>
       <c r="E21" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-3.0810928850663</v>
+        <v>-1.56892791243146</v>
       </c>
       <c r="F21" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-2.0810928850663</v>
+        <v>-0.568927912431465</v>
       </c>
       <c r="G21" s="32" t="n">
         <f aca="false">(G$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-1.0810928850663</v>
+        <v>0.431072087568535</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="31" t="n">
         <f aca="false">B13</f>
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C22" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-8.46055684128203</v>
+        <v>-6.0410928850663</v>
       </c>
       <c r="D22" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-6.50055684128203</v>
+        <v>-4.0810928850663</v>
       </c>
       <c r="E22" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-5.50055684128203</v>
+        <v>-3.0810928850663</v>
       </c>
       <c r="F22" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-4.50055684128203</v>
+        <v>-2.0810928850663</v>
       </c>
       <c r="G22" s="32" t="n">
         <f aca="false">(G$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-3.50055684128203</v>
+        <v>-1.0810928850663</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="31" t="n">
         <f aca="false">B14</f>
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C23" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-10.5775878029708</v>
+        <v>-8.46055684128203</v>
       </c>
       <c r="D23" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-8.61758780297079</v>
+        <v>-6.50055684128203</v>
       </c>
       <c r="E23" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-7.61758780297079</v>
+        <v>-5.50055684128203</v>
       </c>
       <c r="F23" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-6.61758780297079</v>
+        <v>-4.50055684128203</v>
       </c>
       <c r="G23" s="32" t="n">
         <f aca="false">(G$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
+        <v>-3.50055684128203</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="31" t="n">
+        <f aca="false">B15</f>
+        <v>36</v>
+      </c>
+      <c r="C24" s="32" t="n">
+        <f aca="false">(C$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
+        <v>-10.5775878029708</v>
+      </c>
+      <c r="D24" s="32" t="n">
+        <f aca="false">(D$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
+        <v>-8.61758780297079</v>
+      </c>
+      <c r="E24" s="32" t="n">
+        <f aca="false">(E$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
+        <v>-7.61758780297079</v>
+      </c>
+      <c r="F24" s="32" t="n">
+        <f aca="false">(F$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
+        <v>-6.61758780297079</v>
+      </c>
+      <c r="G24" s="32" t="n">
+        <f aca="false">(G$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
         <v>-5.61758780297079</v>
       </c>
     </row>
@@ -2395,7 +2446,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
         <v>91</v>
       </c>
@@ -2412,7 +2463,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
         <v>93</v>
       </c>

</xml_diff>

<commit_message>
Rechner: Marke 4,04 Euro (Faire-Mieten-Modell) entfernt, auch aus Übersicht und Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -323,7 +323,7 @@
     <t xml:space="preserve">Positiv: Überschuss. Negativ (rot): Zuschuss aus dem Landeshaushalt. Im DIW aktuell sind die Vorzeichen umgekehrt.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mieten: 4,04 Faire-Mieten-Modell (Holm et al. 2025) · 6,00 Untergrenze einkommensabhängiger Mieten im kommunalen Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø Miete der landeseigenen Unternehmen · 8,00 ≈ heutiges Niveau in den Beständen.</t>
+    <t xml:space="preserve">Mieten: 6,00 Untergrenze einkommensabhängiger Mieten im kommunalen Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø Miete der landeseigenen Unternehmen · 8,00 ≈ heutiges Niveau in den Beständen.</t>
   </si>
   <si>
     <t xml:space="preserve">Annahmen</t>
@@ -368,7 +368,7 @@
     <t xml:space="preserve">Nettokaltmiete im ersten Jahr</t>
   </si>
   <si>
-    <t xml:space="preserve">4,04 Faire-Mieten-Modell (Holm et al. 2025) · 6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø landeseigene Unternehmen 2025 (7,11; DIW aktuell Nr. 126), Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (DIW aktuell Nr. 126 nach Geschäftsberichten von Adler, Grand City Properties, Vonovia).</t>
+    <t xml:space="preserve">6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø landeseigene Unternehmen 2025 (7,11; DIW aktuell Nr. 126), Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (DIW aktuell Nr. 126 nach Geschäftsberichten von Adler, Grand City Properties, Vonovia).</t>
   </si>
   <si>
     <t xml:space="preserve">Mietsteigerung pro Jahr</t>
@@ -1955,18 +1955,15 @@
         <v>82</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>4.04</v>
+        <v>6</v>
       </c>
       <c r="D8" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F8" s="27" t="n">
-        <v>8</v>
-      </c>
-      <c r="G8" s="27" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1976,22 +1973,18 @@
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B9*$C$5</f>
-        <v>-370.59062782798</v>
+        <v>-26.2578278279798</v>
       </c>
       <c r="D9" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B9*$C$5</f>
-        <v>-26.2578278279798</v>
+        <v>149.42217217202</v>
       </c>
       <c r="E9" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B9*$C$5</f>
-        <v>149.42217217202</v>
+        <v>325.10217217202</v>
       </c>
       <c r="F9" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B9*$C$5</f>
-        <v>325.10217217202</v>
-      </c>
-      <c r="G9" s="29" t="n">
-        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B9*$C$5</f>
         <v>500.78217217202</v>
       </c>
     </row>
@@ -2001,22 +1994,18 @@
       </c>
       <c r="C10" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B10*$C$5</f>
-        <v>-529.984913263472</v>
+        <v>-185.652113263472</v>
       </c>
       <c r="D10" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B10*$C$5</f>
-        <v>-185.652113263472</v>
+        <v>-9.97211326347224</v>
       </c>
       <c r="E10" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B10*$C$5</f>
-        <v>-9.97211326347224</v>
+        <v>165.707886736528</v>
       </c>
       <c r="F10" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B10*$C$5</f>
-        <v>165.707886736528</v>
-      </c>
-      <c r="G10" s="29" t="n">
-        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B10*$C$5</f>
         <v>341.387886736528</v>
       </c>
     </row>
@@ -2026,22 +2015,18 @@
       </c>
       <c r="C11" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B11*$C$5</f>
-        <v>-662.813484459716</v>
+        <v>-318.480684459716</v>
       </c>
       <c r="D11" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B11*$C$5</f>
-        <v>-318.480684459716</v>
+        <v>-142.800684459716</v>
       </c>
       <c r="E11" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B11*$C$5</f>
-        <v>-142.800684459716</v>
+        <v>32.8793155402839</v>
       </c>
       <c r="F11" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B11*$C$5</f>
-        <v>32.8793155402839</v>
-      </c>
-      <c r="G11" s="29" t="n">
-        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B11*$C$5</f>
         <v>208.559315540284</v>
       </c>
     </row>
@@ -2051,22 +2036,18 @@
       </c>
       <c r="C12" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-795.64205565596</v>
+        <v>-451.30925565596</v>
       </c>
       <c r="D12" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-451.30925565596</v>
+        <v>-275.62925565596</v>
       </c>
       <c r="E12" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-275.62925565596</v>
+        <v>-99.9492556559599</v>
       </c>
       <c r="F12" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
-        <v>-99.9492556559599</v>
-      </c>
-      <c r="G12" s="29" t="n">
-        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B12*$C$5</f>
         <v>75.7307443440403</v>
       </c>
     </row>
@@ -2076,22 +2057,18 @@
       </c>
       <c r="C13" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-1061.29919804845</v>
+        <v>-716.966398048447</v>
       </c>
       <c r="D13" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-716.966398048447</v>
+        <v>-541.286398048447</v>
       </c>
       <c r="E13" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-541.286398048447</v>
+        <v>-365.606398048447</v>
       </c>
       <c r="F13" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
-        <v>-365.606398048447</v>
-      </c>
-      <c r="G13" s="29" t="n">
-        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B13*$C$5</f>
         <v>-189.926398048447</v>
       </c>
     </row>
@@ -2101,22 +2078,18 @@
       </c>
       <c r="C14" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-1486.35062587643</v>
+        <v>-1142.01782587643</v>
       </c>
       <c r="D14" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-1142.01782587643</v>
+        <v>-966.337825876427</v>
       </c>
       <c r="E14" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-966.337825876427</v>
+        <v>-790.657825876427</v>
       </c>
       <c r="F14" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
-        <v>-790.657825876427</v>
-      </c>
-      <c r="G14" s="29" t="n">
-        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B14*$C$5</f>
         <v>-614.977825876427</v>
       </c>
     </row>
@@ -2126,22 +2099,18 @@
       </c>
       <c r="C15" s="29" t="n">
         <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-1858.27062522591</v>
+        <v>-1513.93782522591</v>
       </c>
       <c r="D15" s="29" t="n">
         <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-1513.93782522591</v>
+        <v>-1338.25782522591</v>
       </c>
       <c r="E15" s="29" t="n">
         <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-1338.25782522591</v>
+        <v>-1162.57782522591</v>
       </c>
       <c r="F15" s="29" t="n">
         <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-1162.57782522591</v>
-      </c>
-      <c r="G15" s="29" t="n">
-        <f aca="false">(G$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
         <v>-986.897825225909</v>
       </c>
     </row>
@@ -2156,22 +2125,18 @@
       </c>
       <c r="C17" s="30" t="n">
         <f aca="false">C8</f>
-        <v>4.04</v>
+        <v>6</v>
       </c>
       <c r="D17" s="30" t="n">
         <f aca="false">D8</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E17" s="30" t="n">
         <f aca="false">E8</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F17" s="30" t="n">
         <f aca="false">F8</f>
-        <v>8</v>
-      </c>
-      <c r="G17" s="30" t="n">
-        <f aca="false">G8</f>
         <v>9</v>
       </c>
     </row>
@@ -2182,22 +2147,18 @@
       </c>
       <c r="C18" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B18*$C$5*1000000/Flaeche/12)</f>
-        <v>-2.10946395621573</v>
+        <v>-0.149463956215732</v>
       </c>
       <c r="D18" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B18*$C$5*1000000/Flaeche/12)</f>
-        <v>-0.149463956215732</v>
+        <v>0.850536043784268</v>
       </c>
       <c r="E18" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B18*$C$5*1000000/Flaeche/12)</f>
-        <v>0.850536043784268</v>
+        <v>1.85053604378427</v>
       </c>
       <c r="F18" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B18*$C$5*1000000/Flaeche/12)</f>
-        <v>1.85053604378427</v>
-      </c>
-      <c r="G18" s="32" t="n">
-        <f aca="false">(G$17-Bewirtschaftung)-($B18*$C$5*1000000/Flaeche/12)</f>
         <v>2.85053604378427</v>
       </c>
     </row>
@@ -2208,22 +2169,18 @@
       </c>
       <c r="C19" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B19*$C$5*1000000/Flaeche/12)</f>
-        <v>-3.01676293979663</v>
+        <v>-1.05676293979663</v>
       </c>
       <c r="D19" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B19*$C$5*1000000/Flaeche/12)</f>
-        <v>-1.05676293979663</v>
+        <v>-0.0567629397966321</v>
       </c>
       <c r="E19" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B19*$C$5*1000000/Flaeche/12)</f>
-        <v>-0.0567629397966321</v>
+        <v>0.943237060203368</v>
       </c>
       <c r="F19" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B19*$C$5*1000000/Flaeche/12)</f>
-        <v>0.943237060203368</v>
-      </c>
-      <c r="G19" s="32" t="n">
-        <f aca="false">(G$17-Bewirtschaftung)-($B19*$C$5*1000000/Flaeche/12)</f>
         <v>1.94323706020337</v>
       </c>
     </row>
@@ -2234,22 +2191,18 @@
       </c>
       <c r="C20" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B20*$C$5*1000000/Flaeche/12)</f>
-        <v>-3.77284542611405</v>
+        <v>-1.81284542611405</v>
       </c>
       <c r="D20" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B20*$C$5*1000000/Flaeche/12)</f>
-        <v>-1.81284542611405</v>
+        <v>-0.812845426114048</v>
       </c>
       <c r="E20" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B20*$C$5*1000000/Flaeche/12)</f>
-        <v>-0.812845426114048</v>
+        <v>0.187154573885952</v>
       </c>
       <c r="F20" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B20*$C$5*1000000/Flaeche/12)</f>
-        <v>0.187154573885952</v>
-      </c>
-      <c r="G20" s="32" t="n">
-        <f aca="false">(G$17-Bewirtschaftung)-($B20*$C$5*1000000/Flaeche/12)</f>
         <v>1.18715457388595</v>
       </c>
     </row>
@@ -2260,22 +2213,18 @@
       </c>
       <c r="C21" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-4.52892791243147</v>
+        <v>-2.56892791243146</v>
       </c>
       <c r="D21" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-2.56892791243146</v>
+        <v>-1.56892791243146</v>
       </c>
       <c r="E21" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-1.56892791243146</v>
+        <v>-0.568927912431465</v>
       </c>
       <c r="F21" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
-        <v>-0.568927912431465</v>
-      </c>
-      <c r="G21" s="32" t="n">
-        <f aca="false">(G$17-Bewirtschaftung)-($B21*$C$5*1000000/Flaeche/12)</f>
         <v>0.431072087568535</v>
       </c>
     </row>
@@ -2286,22 +2235,18 @@
       </c>
       <c r="C22" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-6.0410928850663</v>
+        <v>-4.0810928850663</v>
       </c>
       <c r="D22" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-4.0810928850663</v>
+        <v>-3.0810928850663</v>
       </c>
       <c r="E22" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-3.0810928850663</v>
+        <v>-2.0810928850663</v>
       </c>
       <c r="F22" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
-        <v>-2.0810928850663</v>
-      </c>
-      <c r="G22" s="32" t="n">
-        <f aca="false">(G$17-Bewirtschaftung)-($B22*$C$5*1000000/Flaeche/12)</f>
         <v>-1.0810928850663</v>
       </c>
     </row>
@@ -2312,22 +2257,18 @@
       </c>
       <c r="C23" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-8.46055684128203</v>
+        <v>-6.50055684128203</v>
       </c>
       <c r="D23" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-6.50055684128203</v>
+        <v>-5.50055684128203</v>
       </c>
       <c r="E23" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-5.50055684128203</v>
+        <v>-4.50055684128203</v>
       </c>
       <c r="F23" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
-        <v>-4.50055684128203</v>
-      </c>
-      <c r="G23" s="32" t="n">
-        <f aca="false">(G$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
         <v>-3.50055684128203</v>
       </c>
     </row>
@@ -2338,22 +2279,18 @@
       </c>
       <c r="C24" s="32" t="n">
         <f aca="false">(C$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-10.5775878029708</v>
+        <v>-8.61758780297079</v>
       </c>
       <c r="D24" s="32" t="n">
         <f aca="false">(D$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-8.61758780297079</v>
+        <v>-7.61758780297079</v>
       </c>
       <c r="E24" s="32" t="n">
         <f aca="false">(E$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-7.61758780297079</v>
+        <v>-6.61758780297079</v>
       </c>
       <c r="F24" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-6.61758780297079</v>
-      </c>
-      <c r="G24" s="32" t="n">
-        <f aca="false">(G$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
         <v>-5.61758780297079</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Rechner: Marken 21 und 36 Mrd. Euro entfernt; Übersicht mit 16 statt 36 Mrd.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -2093,27 +2093,6 @@
         <v>-614.977825876427</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="28" t="n">
-        <v>36</v>
-      </c>
-      <c r="C15" s="29" t="n">
-        <f aca="false">(C$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-1513.93782522591</v>
-      </c>
-      <c r="D15" s="29" t="n">
-        <f aca="false">(D$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-1338.25782522591</v>
-      </c>
-      <c r="E15" s="29" t="n">
-        <f aca="false">(E$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-1162.57782522591</v>
-      </c>
-      <c r="F15" s="29" t="n">
-        <f aca="false">(F$8-Bewirtschaftung)*Flaeche*12/1000000-$B15*$C$5</f>
-        <v>-986.897825225909</v>
-      </c>
-    </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="25" t="s">
         <v>83</v>
@@ -2270,28 +2249,6 @@
       <c r="F23" s="32" t="n">
         <f aca="false">(F$17-Bewirtschaftung)-($B23*$C$5*1000000/Flaeche/12)</f>
         <v>-3.50055684128203</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="31" t="n">
-        <f aca="false">B15</f>
-        <v>36</v>
-      </c>
-      <c r="C24" s="32" t="n">
-        <f aca="false">(C$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-8.61758780297079</v>
-      </c>
-      <c r="D24" s="32" t="n">
-        <f aca="false">(D$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-7.61758780297079</v>
-      </c>
-      <c r="E24" s="32" t="n">
-        <f aca="false">(E$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-6.61758780297079</v>
-      </c>
-      <c r="F24" s="32" t="n">
-        <f aca="false">(F$17-Bewirtschaftung)-($B24*$C$5*1000000/Flaeche/12)</f>
-        <v>-5.61758780297079</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Rechner: Kennzahlen Barwert und höchstes aufgelaufenes Defizit entfernt
Sechs Kennzahlen in drei Spalten; im Excel-Blatt Ergebnis ebenso entfernt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="185">
   <si>
     <t xml:space="preserve">Was kostet die Vergesellschaftung den Berliner Landeshaushalt?</t>
   </si>
@@ -230,364 +230,355 @@
     <t xml:space="preserve">Summe aller Jahressalden</t>
   </si>
   <si>
+    <t xml:space="preserve">Saldo im letzten Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zahl der Jahre mit Zuschuss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dauerhaft ohne Zuschuss ab Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">erstes Jahr, nach dem kein Zuschuss mehr nötig ist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restschuld am Ende des Zeitraums</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schulden des Landes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigenkapitalbedarf des Landes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigenkapitalquote × Entschädigung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anstieg des Schuldenstands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bezogen auf ≈ 69 Mrd. € Schuldenstand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kredite der Anstalt (außerhalb des Landeshaushalts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">solange die Anstalt nicht dem Staatssektor zugerechnet wird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wann trägt sich die Vergesellschaftung im ersten Jahr?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Höchste Entschädigung, die sich bei dieser Miete trägt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mrd. €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reinertrag / [q · AF(Zins Land) + (1 − q) · AF(Zins Anstalt)]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mindestmiete bei dieser Entschädigung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/m² und Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bewirtschaftung + Kapitaldienst je m² und Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix: Saldo im ersten Jahr nach Entschädigung und Miete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zinsen, Eigenkapitalquote, Laufzeiten, Bestand und Bewirtschaftungskosten aus dem Blatt „Annahmen“. Mit den Standardwerten entspricht das Tabelle 2 im DIW aktuell Nr. 126. Zeilen- und Spaltenköpfe (blau) sind änderbar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapitaldienst je Mrd. € Entschädigung (Mio. € pro Jahr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mio. € pro Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entschädigung (Mrd. €) \ Miete (€/m²)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€ je m² Wohnfläche und Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positiv: Überschuss. Negativ (rot): Zuschuss aus dem Landeshaushalt. Im DIW aktuell sind die Vorzeichen umgekehrt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mieten: 6,00 Untergrenze einkommensabhängiger Mieten im kommunalen Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø Miete der landeseigenen Unternehmen · 8,00 ≈ heutiges Niveau in den Beständen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annahmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nur blaue Zellen in Spalte C ändern. Spalte D zeigt den Standardwert des Online-Rechners.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelle / Herleitung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entschädigung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spannweite der Schätzungen 8–36 Mrd. €: Initiative DWE 8/11; Holm et al. (2025) 10,1 (realitätsnah 10–17); IMK (2026) 13,5; Sondierungspapier Linke/Grüne/SPD (Okt. 2026) Obergrenze 16 für rund 160.000 Wohnungen; Rechnungshof Berlin (2024) 8/11/29/36; Senat (2019/20) Verkehrswert 29–36 (bis 39,5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zahl der Wohnungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wohnungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechnungshof Berlin (2024), Holm et al. (2025). Alternativen: IMK / DWE-Gesetzentwurf 2025: 210.000; Sondierungspapier Linke/Grüne/SPD 2026: rund 160.000 (Unternehmen &gt; 10.000 Wohnungen).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø Wohnfläche je Wohnung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechnungshof Berlin (2024). Alternative IMK: 63 m².</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nettokaltmiete im ersten Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø landeseigene Unternehmen 2025 (7,11; DIW aktuell Nr. 126), Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (DIW aktuell Nr. 126 nach Geschäftsberichten von Adler, Grand City Properties, Vonovia).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mietsteigerung pro Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% p.a.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ab dem zweiten Jahr. 1 % wie politisch debattiert (Wahlprogramm Die Linke Berlin 2026: Mieterhöhungen der LWU max. 1 % p.a.; auch Holm et al. 2025, Grundmodell).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bewirtschaftungskosten im ersten Jahr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holm et al. (2025), Tab. 5 (LWU): Instandhaltung 1,77 + Modernisierung 1,00 + Verwaltung 0,52 + Mietausfallwagnis 0,14 + nicht umlagefähige Betriebskosten 0,30. Alternativen: 2,94 (Holm Basis), 3,66 (IMK), 4,40 (IW Köln), 4,44 (Holm Plus).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kostensteigerung pro Jahr (fest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fest: Inflationsziel der EZB. Im Online-Rechner nicht veränderbar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigenkapitalquote (Land, kreditfinanziert)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holm et al. (2025): 20 %; IMK (2026): 30 %.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zins auf den Eigenkapital-Kredit des Landes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30-jährige Bundesanleihe 3,79 % (Bundesbank, 20.10.2026) + Berlin-Aufschlag ≈ 0,2 Prozentpunkte ≈ 4 %.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zins auf die Kredite der Anstalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundesanleihen mittlerer Laufzeit ≈ 3,3 % (Bundesbank, 20.10.2026) + rund 1 Prozentpunkt Aufschlag (HOWOGE-Anleihe, 7 J. Restlaufzeit); 5 % vorsichtig gerundet. Holm et al. (2025): +1,5 bis +2,0 Prozentpunkte. Sensitivität: Zinsen jeweils +1 Pp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laufzeit Eigenkapital-Kredit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIW aktuell: 50 Jahre; IMK: 40; Holm: 30/60/90.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laufzeit Kredite der Anstalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wie oben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tilgungsform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annuität</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annuität / nur Zinsen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">„nur Zinsen“: Kredite werden dauerhaft verlängert, die Schuld bleibt in voller Höhe bestehen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jahre (1–100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Für Summen, Barwert und Zeitreihe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diskontsatz für den Barwert (leer = Zins Land)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leer lassen, um mit dem Zins des Landes zu diskontieren.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abgeleitete Größen (Formeln)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Größe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gesamtwohnfläche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wohnungen × Wohnfläche je Wohnung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigenkapital des Landes (kreditfinanziert)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kredite der Anstalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1 − Eigenkapitalquote) × Entschädigung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nur Zinsen? (1 = ja)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annuitätenfaktor Eigenkapital-Kredit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r / (1 − (1 + r)^−n); bei r = 0: 1/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annuitätenfaktor Kredite der Anstalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapitaldienst Land pro Jahr (solange getilgt wird)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eigenkapital × Annuitätenfaktor (bzw. × Zins)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapitaldienst Anstalt pro Jahr (solange getilgt wird)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fremdkapital × Annuitätenfaktor (bzw. × Zins)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diskontsatz (verwendet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eingabe oder Zins Land</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vergleichsgrößen Landeshaushalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bereinigte Ausgaben des Landes 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doppelhaushalt 2026/27, Pressemitteilung SenFin Nr. 21 vom 19.12.2025; 2026: knapp 45 Mrd. € (wie DIW aktuell Nr. 126)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzierungsdefizit 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statusbericht Senat zur Haushaltslage, 1.9.2026 (Einnahmen 39,1, Ausgaben 43,7 Mrd. €)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einzelplan 10 (Bildung, Jugend, Familie) 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doppelhaushalt 2026/27; ohne die Schulausgaben der Bezirke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Struktureller Verschuldungsspielraum (Obergrenze)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,35 % BIP, Länderanteil; Schätzung 675–800 Mio. € p.a. (Tagesspiegel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schuldenstand des Landes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senatsverwaltung für Finanzen; steigt bis 2027 auf über 75 Mrd. €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeitreihe: Rechnung Jahr für Jahr (Mio. € pro Jahr, nominal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeilen jenseits des Betrachtungszeitraums bleiben leer. Saldo positiv = Überschuss, negativ = Zuschuss aus dem Landeshaushalt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Im Zeitraum (1 = ja)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Miete €/m²/Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bewirtschaftung €/m²/Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mieteinnahmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bewirtschaftungskosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reinertrag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapitaldienst Land (EK-Kredit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapitaldienst gesamt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo Landeshaushalt (+ Überschuss, − Zuschuss)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo €/m²/Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo € je Wohnung/Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo kumuliert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo Anstalt (Reinertrag − KD Anstalt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restschuld EK-Kredit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restschuld Anstalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diskontfaktor</t>
+  </si>
+  <si>
     <t xml:space="preserve">Barwert des Saldos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">abgezinst mit dem Diskontsatz (Blatt Annahmen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo im letzten Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maximales kumuliertes Defizit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tiefster Stand des aufsummierten Saldos, als Betrag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zahl der Jahre mit Zuschuss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dauerhaft ohne Zuschuss ab Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">erstes Jahr, nach dem kein Zuschuss mehr nötig ist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restschuld am Ende des Zeitraums</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schulden des Landes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eigenkapitalbedarf des Landes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eigenkapitalquote × Entschädigung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anstieg des Schuldenstands</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bezogen auf ≈ 69 Mrd. € Schuldenstand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kredite der Anstalt (außerhalb des Landeshaushalts)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">solange die Anstalt nicht dem Staatssektor zugerechnet wird</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wann trägt sich die Vergesellschaftung im ersten Jahr?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Höchste Entschädigung, die sich bei dieser Miete trägt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mrd. €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reinertrag / [q · AF(Zins Land) + (1 − q) · AF(Zins Anstalt)]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mindestmiete bei dieser Entschädigung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€/m² und Monat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bewirtschaftung + Kapitaldienst je m² und Monat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matrix: Saldo im ersten Jahr nach Entschädigung und Miete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zinsen, Eigenkapitalquote, Laufzeiten, Bestand und Bewirtschaftungskosten aus dem Blatt „Annahmen“. Mit den Standardwerten entspricht das Tabelle 2 im DIW aktuell Nr. 126. Zeilen- und Spaltenköpfe (blau) sind änderbar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kapitaldienst je Mrd. € Entschädigung (Mio. € pro Jahr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mio. € pro Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entschädigung (Mrd. €) \ Miete (€/m²)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€ je m² Wohnfläche und Monat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Positiv: Überschuss. Negativ (rot): Zuschuss aus dem Landeshaushalt. Im DIW aktuell sind die Vorzeichen umgekehrt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mieten: 6,00 Untergrenze einkommensabhängiger Mieten im kommunalen Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø Miete der landeseigenen Unternehmen · 8,00 ≈ heutiges Niveau in den Beständen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annahmen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nur blaue Zellen in Spalte C ändern. Spalte D zeigt den Standardwert des Online-Rechners.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Standard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelle / Herleitung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entschädigung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spannweite der Schätzungen 8–36 Mrd. €: Initiative DWE 8/11; Holm et al. (2025) 10,1 (realitätsnah 10–17); IMK (2026) 13,5; Sondierungspapier Linke/Grüne/SPD (Okt. 2026) Obergrenze 16 für rund 160.000 Wohnungen; Rechnungshof Berlin (2024) 8/11/29/36; Senat (2019/20) Verkehrswert 29–36 (bis 39,5).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zahl der Wohnungen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wohnungen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rechnungshof Berlin (2024), Holm et al. (2025). Alternativen: IMK / DWE-Gesetzentwurf 2025: 210.000; Sondierungspapier Linke/Grüne/SPD 2026: rund 160.000 (Unternehmen &gt; 10.000 Wohnungen).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ø Wohnfläche je Wohnung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rechnungshof Berlin (2024). Alternative IMK: 63 m².</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nettokaltmiete im ersten Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,00 Untergrenze einkommensabh. Mieten kommunaler Neubau (Wahlprogramm Die Linke 2026) · 7,00 ≈ Ø landeseigene Unternehmen 2025 (7,11; DIW aktuell Nr. 126), Grundmodell Holm et al. · 7,08 Ø LWU (IMK 2026) · ≈ 8,00 heutiges Niveau in den Beständen (DIW aktuell Nr. 126 nach Geschäftsberichten von Adler, Grand City Properties, Vonovia).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mietsteigerung pro Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% p.a.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ab dem zweiten Jahr. 1 % wie politisch debattiert (Wahlprogramm Die Linke Berlin 2026: Mieterhöhungen der LWU max. 1 % p.a.; auch Holm et al. 2025, Grundmodell).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bewirtschaftungskosten im ersten Jahr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holm et al. (2025), Tab. 5 (LWU): Instandhaltung 1,77 + Modernisierung 1,00 + Verwaltung 0,52 + Mietausfallwagnis 0,14 + nicht umlagefähige Betriebskosten 0,30. Alternativen: 2,94 (Holm Basis), 3,66 (IMK), 4,40 (IW Köln), 4,44 (Holm Plus).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kostensteigerung pro Jahr (fest)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fest: Inflationsziel der EZB. Im Online-Rechner nicht veränderbar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eigenkapitalquote (Land, kreditfinanziert)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anteil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holm et al. (2025): 20 %; IMK (2026): 30 %.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zins auf den Eigenkapital-Kredit des Landes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30-jährige Bundesanleihe 3,79 % (Bundesbank, 20.10.2026) + Berlin-Aufschlag ≈ 0,2 Prozentpunkte ≈ 4 %.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zins auf die Kredite der Anstalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bundesanleihen mittlerer Laufzeit ≈ 3,3 % (Bundesbank, 20.10.2026) + rund 1 Prozentpunkt Aufschlag (HOWOGE-Anleihe, 7 J. Restlaufzeit); 5 % vorsichtig gerundet. Holm et al. (2025): +1,5 bis +2,0 Prozentpunkte. Sensitivität: Zinsen jeweils +1 Pp.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laufzeit Eigenkapital-Kredit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIW aktuell: 50 Jahre; IMK: 40; Holm: 30/60/90.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laufzeit Kredite der Anstalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wie oben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tilgungsform</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annuität</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annuität / nur Zinsen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">„nur Zinsen“: Kredite werden dauerhaft verlängert, die Schuld bleibt in voller Höhe bestehen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jahre (1–100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Für Summen, Barwert und Zeitreihe.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diskontsatz für den Barwert (leer = Zins Land)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leer lassen, um mit dem Zins des Landes zu diskontieren.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abgeleitete Größen (Formeln)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Größe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gesamtwohnfläche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wohnungen × Wohnfläche je Wohnung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eigenkapital des Landes (kreditfinanziert)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kredite der Anstalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1 − Eigenkapitalquote) × Entschädigung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nur Zinsen? (1 = ja)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annuitätenfaktor Eigenkapital-Kredit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">r / (1 − (1 + r)^−n); bei r = 0: 1/n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annuitätenfaktor Kredite der Anstalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kapitaldienst Land pro Jahr (solange getilgt wird)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eigenkapital × Annuitätenfaktor (bzw. × Zins)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kapitaldienst Anstalt pro Jahr (solange getilgt wird)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fremdkapital × Annuitätenfaktor (bzw. × Zins)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diskontsatz (verwendet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eingabe oder Zins Land</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vergleichsgrößen Landeshaushalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bereinigte Ausgaben des Landes 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doppelhaushalt 2026/27, Pressemitteilung SenFin Nr. 21 vom 19.12.2025; 2026: knapp 45 Mrd. € (wie DIW aktuell Nr. 126)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzierungsdefizit 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Statusbericht Senat zur Haushaltslage, 1.9.2026 (Einnahmen 39,1, Ausgaben 43,7 Mrd. €)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einzelplan 10 (Bildung, Jugend, Familie) 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doppelhaushalt 2026/27; ohne die Schulausgaben der Bezirke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Struktureller Verschuldungsspielraum (Obergrenze)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,35 % BIP, Länderanteil; Schätzung 675–800 Mio. € p.a. (Tagesspiegel)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schuldenstand des Landes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Senatsverwaltung für Finanzen; steigt bis 2027 auf über 75 Mrd. €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zeitreihe: Rechnung Jahr für Jahr (Mio. € pro Jahr, nominal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zeilen jenseits des Betrachtungszeitraums bleiben leer. Saldo positiv = Überschuss, negativ = Zuschuss aus dem Landeshaushalt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Im Zeitraum (1 = ja)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Miete €/m²/Monat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bewirtschaftung €/m²/Monat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mieteinnahmen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bewirtschaftungskosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reinertrag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kapitaldienst Land (EK-Kredit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kapitaldienst gesamt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo Landeshaushalt (+ Überschuss, − Zuschuss)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo €/m²/Monat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo € je Wohnung/Monat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo kumuliert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo Anstalt (Reinertrag − KD Anstalt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restschuld EK-Kredit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restschuld Anstalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diskontfaktor</t>
   </si>
   <si>
     <t xml:space="preserve">Jahr mit Zuschuss</t>
@@ -1447,7 +1438,7 @@
     <tabColor rgb="FF6FC8B6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:E37"/>
+  <dimension ref="B1:E35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1714,39 +1705,37 @@
         <v>54</v>
       </c>
       <c r="C23" s="16" t="n">
-        <f aca="false">SUM(Z_Barwert)</f>
-        <v>-4258.15411069692</v>
+        <f aca="false">INDEX(Z_Saldo_LH,Horizont)</f>
+        <v>-443.974112005765</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="13" t="s">
-        <v>55</v>
-      </c>
+      <c r="E23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24" s="16" t="n">
-        <f aca="false">INDEX(Z_Saldo_LH,Horizont)</f>
-        <v>-443.974112005765</v>
+        <v>55</v>
+      </c>
+      <c r="C24" s="19" t="n">
+        <f aca="false">COUNT(Z_MitZuschuss)</f>
+        <v>50</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="E24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="19" t="str">
+        <f aca="false">IF(COUNT(Z_MitZuschuss)=0,1,IF(MAX(Z_MitZuschuss)&gt;=Horizont,"nicht im Zeitraum",MAX(Z_MitZuschuss)+1))</f>
+        <v>nicht im Zeitraum</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>57</v>
-      </c>
-      <c r="C25" s="15" t="n">
-        <f aca="false">MAX(0,-MIN(Z_Kum))</f>
-        <v>12013.2027926495</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>26</v>
       </c>
       <c r="E25" s="13" t="s">
         <v>58</v>
@@ -1756,55 +1745,57 @@
       <c r="B26" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="19" t="n">
-        <f aca="false">COUNT(Z_MitZuschuss)</f>
-        <v>50</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="E26" s="13"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" s="19" t="str">
-        <f aca="false">IF(COUNT(Z_MitZuschuss)=0,1,IF(MAX(Z_MitZuschuss)&gt;=Horizont,"nicht im Zeitraum",MAX(Z_MitZuschuss)+1))</f>
-        <v>nicht im Zeitraum</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="15" t="n">
+      <c r="C26" s="15" t="n">
         <f aca="false">INDEX(Z_RestEK,Horizont)+INDEX(Z_RestFK,Horizont)</f>
         <v>0</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="D26" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="13"/>
+      <c r="E26" s="13"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <f aca="false">Eigenkapital</f>
+        <v>2700</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="20" t="n">
+        <f aca="false">Eigenkapital/HH_Schulden</f>
+        <v>0.0391304347826087</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="13" t="s">
         <v>64</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1812,8 +1803,8 @@
         <v>65</v>
       </c>
       <c r="C31" s="15" t="n">
-        <f aca="false">Eigenkapital</f>
-        <v>2700</v>
+        <f aca="false">Fremdkapital</f>
+        <v>10800</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>26</v>
@@ -1822,78 +1813,48 @@
         <v>66</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="12" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="20" t="n">
-        <f aca="false">Eigenkapital/HH_Schulden</f>
-        <v>0.0391304347826087</v>
-      </c>
-      <c r="D32" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E32" s="13" t="s">
+      <c r="C33" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="12" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="C33" s="15" t="n">
-        <f aca="false">Fremdkapital</f>
-        <v>10800</v>
-      </c>
-      <c r="D33" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="C36" s="21" t="n">
+      <c r="C34" s="21" t="n">
         <f aca="false">MAX(0,Zeitreihe!G5)/1000/(EK_Quote*IF(Nur_Zinsen=1,Zins_EK,AF_EK)+(1-EK_Quote)*IF(Nur_Zinsen=1,Zins_FK,AF_FK))</f>
         <v>10.8123123441428</v>
       </c>
-      <c r="D36" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" s="22" t="n">
+      <c r="D34" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="22" t="n">
         <f aca="false">Bewirtschaftung+Zeitreihe!J5*1000000/Flaeche/12</f>
         <v>7.81284542611405</v>
       </c>
-      <c r="D37" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>77</v>
+      <c r="D35" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1922,12 +1883,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1938,7 +1899,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C5" s="24" t="n">
         <f aca="false">1000*(EK_Quote*IF(Nur_Zinsen=1,Zins_EK,AF_EK)+(1-EK_Quote)*IF(Nur_Zinsen=1,Zins_FK,AF_FK))</f>
@@ -1947,12 +1908,12 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="25" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C8" s="27" t="n">
         <v>6</v>
@@ -2095,12 +2056,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="25" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C17" s="30" t="n">
         <f aca="false">C8</f>
@@ -2253,12 +2214,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="33" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C26" s="33"/>
       <c r="D26" s="33"/>
@@ -2315,34 +2276,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>23</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C5" s="34" t="n">
         <v>13.5</v>
@@ -2351,15 +2312,15 @@
         <v>13.5</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C6" s="37" t="n">
         <v>240000</v>
@@ -2368,15 +2329,15 @@
         <v>240000</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="12" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C7" s="37" t="n">
         <v>61</v>
@@ -2385,15 +2346,15 @@
         <v>61</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C8" s="39" t="n">
         <v>7</v>
@@ -2402,15 +2363,15 @@
         <v>7</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F8" s="36" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="12" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C9" s="41" t="n">
         <v>0.01</v>
@@ -2419,15 +2380,15 @@
         <v>0.01</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F9" s="36" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="12" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C10" s="43" t="n">
         <v>3.73</v>
@@ -2436,15 +2397,15 @@
         <v>3.73</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="12" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C11" s="20" t="n">
         <v>0.02</v>
@@ -2453,15 +2414,15 @@
         <v>0.02</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F11" s="36" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C12" s="44" t="n">
         <v>0.2</v>
@@ -2470,15 +2431,15 @@
         <v>0.2</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="12" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C13" s="45" t="n">
         <v>0.04</v>
@@ -2487,15 +2448,15 @@
         <v>0.04</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F13" s="36" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C14" s="45" t="n">
         <v>0.05</v>
@@ -2504,15 +2465,15 @@
         <v>0.05</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C15" s="47" t="n">
         <v>50</v>
@@ -2524,12 +2485,12 @@
         <v>49</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="12" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C16" s="47" t="n">
         <v>50</v>
@@ -2541,24 +2502,24 @@
         <v>49</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D17" s="50" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2572,33 +2533,33 @@
         <v>50</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C19" s="51"/>
       <c r="D19" s="46"/>
       <c r="E19" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="25" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>22</v>
@@ -2613,22 +2574,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="12" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C23" s="15" t="n">
         <f aca="false">Wohnungen*Flaeche_je_WE</f>
         <v>14640000</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="12" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C24" s="15" t="n">
         <f aca="false">EK_Quote*Entschaedigung*1000</f>
@@ -2638,12 +2599,12 @@
         <v>26</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="12" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C25" s="15" t="n">
         <f aca="false">(1-EK_Quote)*Entschaedigung*1000</f>
@@ -2653,12 +2614,12 @@
         <v>26</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="12" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C26" s="19" t="n">
         <f aca="false">IF(Tilgung="nur Zinsen",1,0)</f>
@@ -2669,7 +2630,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="12" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C27" s="52" t="n">
         <f aca="false">IF(Zins_EK=0,1/Laufzeit_EK,Zins_EK/(1-(1+Zins_EK)^(-Laufzeit_EK)))</f>
@@ -2677,12 +2638,12 @@
       </c>
       <c r="E27" s="12"/>
       <c r="F27" s="13" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="12" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C28" s="52" t="n">
         <f aca="false">IF(Zins_FK=0,1/Laufzeit_FK,Zins_FK/(1-(1+Zins_FK)^(-Laufzeit_FK)))</f>
@@ -2690,12 +2651,12 @@
       </c>
       <c r="E28" s="12"/>
       <c r="F28" s="13" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="12" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C29" s="21" t="n">
         <f aca="false">Eigenkapital*IF(Nur_Zinsen=1,Zins_EK,AF_EK)</f>
@@ -2705,12 +2666,12 @@
         <v>26</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="12" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C30" s="21" t="n">
         <f aca="false">Fremdkapital*IF(Nur_Zinsen=1,Zins_FK,AF_FK)</f>
@@ -2720,32 +2681,32 @@
         <v>26</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="12" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C31" s="53" t="n">
         <f aca="false">IF(ISBLANK(Diskont_Eingabe),Zins_EK,Diskont_Eingabe)</f>
         <v>0.04</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="25" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>22</v>
@@ -2755,12 +2716,12 @@
         <v>23</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="12" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C35" s="37" t="n">
         <v>45900</v>
@@ -2769,12 +2730,12 @@
         <v>26</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="12" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C36" s="37" t="n">
         <v>4600</v>
@@ -2783,12 +2744,12 @@
         <v>26</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C37" s="37" t="n">
         <v>5430</v>
@@ -2797,12 +2758,12 @@
         <v>26</v>
       </c>
       <c r="F37" s="36" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="12" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C38" s="37" t="n">
         <v>800</v>
@@ -2811,12 +2772,12 @@
         <v>26</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C39" s="37" t="n">
         <v>69000</v>
@@ -2825,7 +2786,7 @@
         <v>26</v>
       </c>
       <c r="F39" s="36" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -2879,74 +2840,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="54" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B4" s="54" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="D4" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="F4" s="54" t="s">
         <v>158</v>
       </c>
-      <c r="C4" s="54" t="s">
+      <c r="G4" s="54" t="s">
         <v>159</v>
       </c>
-      <c r="D4" s="54" t="s">
+      <c r="H4" s="54" t="s">
         <v>160</v>
-      </c>
-      <c r="E4" s="54" t="s">
-        <v>161</v>
-      </c>
-      <c r="F4" s="54" t="s">
-        <v>162</v>
-      </c>
-      <c r="G4" s="54" t="s">
-        <v>163</v>
-      </c>
-      <c r="H4" s="54" t="s">
-        <v>164</v>
       </c>
       <c r="I4" s="54" t="s">
         <v>37</v>
       </c>
       <c r="J4" s="54" t="s">
+        <v>161</v>
+      </c>
+      <c r="K4" s="54" t="s">
+        <v>162</v>
+      </c>
+      <c r="L4" s="54" t="s">
+        <v>163</v>
+      </c>
+      <c r="M4" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="N4" s="54" t="s">
         <v>165</v>
       </c>
-      <c r="K4" s="54" t="s">
+      <c r="O4" s="54" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="54" t="s">
+      <c r="P4" s="54" t="s">
         <v>167</v>
       </c>
-      <c r="M4" s="54" t="s">
+      <c r="Q4" s="54" t="s">
         <v>168</v>
       </c>
-      <c r="N4" s="54" t="s">
+      <c r="R4" s="54" t="s">
         <v>169</v>
       </c>
-      <c r="O4" s="54" t="s">
+      <c r="S4" s="54" t="s">
         <v>170</v>
       </c>
-      <c r="P4" s="54" t="s">
+      <c r="T4" s="54" t="s">
         <v>171</v>
-      </c>
-      <c r="Q4" s="54" t="s">
-        <v>172</v>
-      </c>
-      <c r="R4" s="54" t="s">
-        <v>173</v>
-      </c>
-      <c r="S4" s="54" t="s">
-        <v>54</v>
-      </c>
-      <c r="T4" s="54" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11173,67 +11134,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rechner: Kennzahl Barwert des Saldos wieder aufgenommen (Seite und Excel)
Vier Kennzahlen, auf schmaleren Bildschirmen zwei bzw. eine Spalte.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192eWt6S3uboNKq5nb9mRkk
</commit_message>
<xml_diff>
--- a/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
+++ b/static/vergesellschaftung/Vergesellschaftung_Rechner.xlsx
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="173">
   <si>
     <t xml:space="preserve">Was kostet die Vergesellschaftung den Berliner Landeshaushalt?</t>
   </si>
@@ -222,6 +222,12 @@
     <t xml:space="preserve">Summe aller Jahressalden</t>
   </si>
   <si>
+    <t xml:space="preserve">Barwert des Saldos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abgezinst mit dem Diskontsatz (Blatt Annahmen)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Saldo im letzten Jahr</t>
   </si>
   <si>
@@ -535,9 +541,6 @@
   </si>
   <si>
     <t xml:space="preserve">Diskontfaktor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barwert des Saldos</t>
   </si>
   <si>
     <t xml:space="preserve">Jahr mit Zuschuss</t>
@@ -1392,7 +1395,7 @@
     <tabColor rgb="FF6FC8B6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:E27"/>
+  <dimension ref="B1:E28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1633,84 +1636,99 @@
         <v>52</v>
       </c>
       <c r="C21" s="16" t="n">
+        <f aca="false">SUM(Z_Barwert)</f>
+        <v>-4258.15411069692</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="16" t="n">
         <f aca="false">INDEX(Z_Saldo_LH,Horizont)</f>
         <v>-443.974112005765</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D22" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="13"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="18" t="n">
+      <c r="E22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="18" t="n">
         <f aca="false">COUNT(Z_MitZuschuss)</f>
         <v>50</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D23" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="13"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="18" t="str">
+      <c r="E23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="18" t="str">
         <f aca="false">IF(COUNT(Z_MitZuschuss)=0,1,IF(MAX(Z_MitZuschuss)&gt;=Horizont,"nicht im Zeitraum",MAX(Z_MitZuschuss)+1))</f>
         <v>nicht im Zeitraum</v>
       </c>
-      <c r="D23" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="8" t="s">
+      <c r="D24" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="E24" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E26" s="9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" s="19" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="19" t="n">
         <f aca="false">MAX(0,Zeitreihe!G5)/1000/(EK_Quote*IF(Nur_Zinsen=1,Zins_EK,AF_EK)+(1-EK_Quote)*IF(Nur_Zinsen=1,Zins_FK,AF_FK))</f>
         <v>10.8123123441428</v>
       </c>
-      <c r="D26" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="12" t="s">
+      <c r="D27" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="20" t="n">
+      <c r="E27" s="13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="20" t="n">
         <f aca="false">Bewirtschaftung+Zeitreihe!J5*1000000/Flaeche/12</f>
         <v>7.81284542611405</v>
       </c>
-      <c r="D27" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>63</v>
+      <c r="D28" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1739,12 +1757,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1755,7 +1773,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C5" s="22" t="n">
         <f aca="false">1000*(EK_Quote*IF(Nur_Zinsen=1,Zins_EK,AF_EK)+(1-EK_Quote)*IF(Nur_Zinsen=1,Zins_FK,AF_FK))</f>
@@ -1764,12 +1782,12 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="23" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="24" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C8" s="25" t="n">
         <v>6</v>
@@ -1912,12 +1930,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="23" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="24" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C17" s="28" t="n">
         <f aca="false">C8</f>
@@ -2070,12 +2088,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="31" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C26" s="31"/>
       <c r="D26" s="31"/>
@@ -2132,34 +2150,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>23</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C5" s="32" t="n">
         <v>13.5</v>
@@ -2168,15 +2186,15 @@
         <v>13.5</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F5" s="34" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C6" s="35" t="n">
         <v>240000</v>
@@ -2185,15 +2203,15 @@
         <v>240000</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F6" s="34" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C7" s="35" t="n">
         <v>61</v>
@@ -2202,15 +2220,15 @@
         <v>61</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F7" s="34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C8" s="37" t="n">
         <v>7</v>
@@ -2219,15 +2237,15 @@
         <v>7</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F8" s="34" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C9" s="39" t="n">
         <v>0.01</v>
@@ -2236,15 +2254,15 @@
         <v>0.01</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F9" s="34" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C10" s="41" t="n">
         <v>3.73</v>
@@ -2253,15 +2271,15 @@
         <v>3.73</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F10" s="34" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C11" s="42" t="n">
         <v>0.02</v>
@@ -2270,15 +2288,15 @@
         <v>0.02</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F11" s="34" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C12" s="43" t="n">
         <v>0.2</v>
@@ -2287,15 +2305,15 @@
         <v>0.2</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F12" s="34" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C13" s="44" t="n">
         <v>0.04</v>
@@ -2304,15 +2322,15 @@
         <v>0.04</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F13" s="34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C14" s="44" t="n">
         <v>0.05</v>
@@ -2321,15 +2339,15 @@
         <v>0.05</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F14" s="34" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C15" s="46" t="n">
         <v>50</v>
@@ -2341,12 +2359,12 @@
         <v>47</v>
       </c>
       <c r="F15" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C16" s="46" t="n">
         <v>50</v>
@@ -2358,24 +2376,24 @@
         <v>47</v>
       </c>
       <c r="F16" s="34" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C17" s="48" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D17" s="49" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F17" s="34" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2389,33 +2407,33 @@
         <v>50</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F18" s="34" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="45"/>
       <c r="E19" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F19" s="34" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>22</v>
@@ -2430,22 +2448,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C23" s="15" t="n">
         <f aca="false">Wohnungen*Flaeche_je_WE</f>
         <v>14640000</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C24" s="15" t="n">
         <f aca="false">EK_Quote*Entschaedigung*1000</f>
@@ -2455,12 +2473,12 @@
         <v>26</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="12" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C25" s="15" t="n">
         <f aca="false">(1-EK_Quote)*Entschaedigung*1000</f>
@@ -2470,12 +2488,12 @@
         <v>26</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C26" s="18" t="n">
         <f aca="false">IF(Tilgung="nur Zinsen",1,0)</f>
@@ -2486,7 +2504,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C27" s="51" t="n">
         <f aca="false">IF(Zins_EK=0,1/Laufzeit_EK,Zins_EK/(1-(1+Zins_EK)^(-Laufzeit_EK)))</f>
@@ -2494,12 +2512,12 @@
       </c>
       <c r="E27" s="12"/>
       <c r="F27" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C28" s="51" t="n">
         <f aca="false">IF(Zins_FK=0,1/Laufzeit_FK,Zins_FK/(1-(1+Zins_FK)^(-Laufzeit_FK)))</f>
@@ -2507,12 +2525,12 @@
       </c>
       <c r="E28" s="12"/>
       <c r="F28" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C29" s="19" t="n">
         <f aca="false">Eigenkapital*IF(Nur_Zinsen=1,Zins_EK,AF_EK)</f>
@@ -2522,12 +2540,12 @@
         <v>26</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C30" s="19" t="n">
         <f aca="false">Fremdkapital*IF(Nur_Zinsen=1,Zins_FK,AF_FK)</f>
@@ -2537,32 +2555,32 @@
         <v>26</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C31" s="52" t="n">
         <f aca="false">IF(ISBLANK(Diskont_Eingabe),Zins_EK,Diskont_Eingabe)</f>
         <v>0.04</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="23" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>22</v>
@@ -2572,12 +2590,12 @@
         <v>23</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C35" s="35" t="n">
         <v>45900</v>
@@ -2586,12 +2604,12 @@
         <v>26</v>
       </c>
       <c r="F35" s="34" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C36" s="35" t="n">
         <v>4600</v>
@@ -2600,12 +2618,12 @@
         <v>26</v>
       </c>
       <c r="F36" s="34" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C37" s="35" t="n">
         <v>69000</v>
@@ -2614,7 +2632,7 @@
         <v>26</v>
       </c>
       <c r="F37" s="34" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -2668,74 +2686,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="53" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C4" s="53" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D4" s="53" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E4" s="53" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F4" s="53" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G4" s="53" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H4" s="53" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I4" s="53" t="s">
         <v>37</v>
       </c>
       <c r="J4" s="53" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="K4" s="53" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="L4" s="53" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="M4" s="53" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="N4" s="53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="O4" s="53" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="P4" s="53" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q4" s="53" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="R4" s="53" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="S4" s="53" t="s">
-        <v>157</v>
+        <v>52</v>
       </c>
       <c r="T4" s="53" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10962,67 +10980,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>